<commit_message>
feat: refaktoryzacja kodu i obsluga wielu walut (PLN, EUR, USD, GBP) v2.0
</commit_message>
<xml_diff>
--- a/tests/testy_PL_TEKST.xlsx
+++ b/tests/testy_PL_TEKST.xlsx
@@ -5,15 +5,18 @@
   <workbookPr codeName="Ten_skoroszyt"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Praca\Projekty\repos\PL-TEKST\PL-TEKST\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB20A389-9062-4FE0-99AD-D88C1107AECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_E3A5318B44418F991E720E7711418D457B6691C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Testy PL_TEKST" sheetId="1" r:id="rId1"/>
+    <sheet name="PLN" sheetId="1" r:id="rId1"/>
+    <sheet name="EUR" sheetId="2" r:id="rId2"/>
+    <sheet name="USD" sheetId="3" r:id="rId3"/>
+    <sheet name="GBP" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,12 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
-  <si>
-    <t>Testy edge-case — funkcja PL_TEKST</t>
-  </si>
-  <si>
-    <t>Kolumna D = wynik formuły  |  Kolumna E = oczekiwany wynik  |  Kolumna F = status (OK / SPRAWDŹ)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="98">
+  <si>
+    <t>Testy PLN — funkcja PL_TEKST</t>
+  </si>
+  <si>
+    <t>Kolumna D = wynik formuły  |  Kolumna E = oczekiwany wynik  |  Kolumna F = status</t>
   </si>
   <si>
     <t>#</t>
@@ -210,6 +213,123 @@
   </si>
   <si>
     <t>testów OK</t>
+  </si>
+  <si>
+    <t>Testy EUR — funkcja PL_TEKST</t>
+  </si>
+  <si>
+    <t>Jeden euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwa euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Pięć euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Jedenaście euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwanaście euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwadzieścia jeden euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Sto euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Tysiąc euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwa tysiące euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Tysiąc dwieście trzydzieści cztery euro (67/100 centów)</t>
+  </si>
+  <si>
+    <t>Zero euro (01/100 centów)</t>
+  </si>
+  <si>
+    <t>Zero euro (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Testy USD — funkcja PL_TEKST</t>
+  </si>
+  <si>
+    <t>Jeden dolar (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwa dolary (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Pięć dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Jedenaście dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwanaście dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwadzieścia jeden dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Sto dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Tysiąc dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Dwa tysiące dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Tysiąc dwieście trzydzieści cztery dolary (67/100 centów)</t>
+  </si>
+  <si>
+    <t>Zero dolarów (01/100 centów)</t>
+  </si>
+  <si>
+    <t>Zero dolarów (00/100 centów)</t>
+  </si>
+  <si>
+    <t>Testy GBP — funkcja PL_TEKST</t>
+  </si>
+  <si>
+    <t>Jeden funt (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Dwa funty (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Pięć funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Jedenaście funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Dwanaście funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Dwadzieścia jeden funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Sto funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Tysiąc funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Dwa tysiące funtów (00/100 pensów)</t>
+  </si>
+  <si>
+    <t>Tysiąc dwieście trzydzieści cztery funty (67/100 pensów)</t>
+  </si>
+  <si>
+    <t>Zero funtów (01/100 pensów)</t>
+  </si>
+  <si>
+    <t>Zero funtów (00/100 pensów)</t>
   </si>
 </sst>
 </file>
@@ -357,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -365,9 +485,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -383,11 +501,12 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -408,33 +527,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -745,42 +837,44 @@
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="55" customWidth="1"/>
+    <col min="4" max="5" width="58" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -788,113 +882,113 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="4">
         <v>0</v>
       </c>
-      <c r="D4" s="23" t="str">
-        <f t="shared" ref="D4:D43" si="0">PL_TEKST(C4)</f>
-        <v>Zero złotych (00/100 groszy)</v>
-      </c>
-      <c r="E4" s="24" t="s">
+      <c r="D4" s="5" t="e">
+        <f t="shared" ref="D4:D43" ca="1" si="0">PL_TEKST(C4)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="7" t="str">
-        <f t="shared" ref="F4:F43" si="1">IF(D4=E4,"✅ OK","❌ SPRAWDŹ")</f>
-        <v>✅ OK</v>
+      <c r="F4" s="7" t="e">
+        <f t="shared" ref="F4:F43" ca="1" si="1">IF(D4=E4,"✅ OK","❌ SPRAWDŹ")</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="27">
+      <c r="C5" s="10">
         <v>1</v>
       </c>
-      <c r="D5" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Jeden złoty (00/100 groszy)</v>
-      </c>
-      <c r="E5" s="24" t="s">
+      <c r="D5" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F5" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="4">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwa złote (00/100 groszy)</v>
-      </c>
-      <c r="E6" s="24" t="s">
+      <c r="D6" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F6" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="8">
         <v>4</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="27">
+      <c r="C7" s="10">
         <v>5</v>
       </c>
-      <c r="D7" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Pięć złotych (00/100 groszy)</v>
-      </c>
-      <c r="E7" s="24" t="s">
+      <c r="D7" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F7" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+      <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="4">
         <v>9</v>
       </c>
-      <c r="D8" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziewięć złotych (00/100 groszy)</v>
-      </c>
-      <c r="E8" s="24" t="s">
+      <c r="D8" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F8" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -907,16 +1001,16 @@
       <c r="C9" s="10">
         <v>10</v>
       </c>
-      <c r="D9" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziesięć złotych (00/100 groszy)</v>
+      <c r="D9" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F9" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -929,16 +1023,16 @@
       <c r="C10" s="4">
         <v>11</v>
       </c>
-      <c r="D10" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Jedenaście złotych (00/100 groszy)</v>
+      <c r="D10" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F10" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -951,16 +1045,16 @@
       <c r="C11" s="10">
         <v>12</v>
       </c>
-      <c r="D11" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwanaście złotych (00/100 groszy)</v>
+      <c r="D11" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F11" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -973,16 +1067,16 @@
       <c r="C12" s="4">
         <v>13</v>
       </c>
-      <c r="D12" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Trzynaście złotych (00/100 groszy)</v>
+      <c r="D12" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F12" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -995,16 +1089,16 @@
       <c r="C13" s="10">
         <v>19</v>
       </c>
-      <c r="D13" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziewiętnaście złotych (00/100 groszy)</v>
+      <c r="D13" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F13" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1017,16 +1111,16 @@
       <c r="C14" s="4">
         <v>20</v>
       </c>
-      <c r="D14" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwadzieścia złotych (00/100 groszy)</v>
+      <c r="D14" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F14" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1039,16 +1133,16 @@
       <c r="C15" s="10">
         <v>21</v>
       </c>
-      <c r="D15" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwadzieścia jeden złotych (00/100 groszy)</v>
+      <c r="D15" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F15" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1061,16 +1155,16 @@
       <c r="C16" s="4">
         <v>22</v>
       </c>
-      <c r="D16" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwadzieścia dwa złote (00/100 groszy)</v>
+      <c r="D16" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F16" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1083,16 +1177,16 @@
       <c r="C17" s="10">
         <v>99</v>
       </c>
-      <c r="D17" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziewięćdziesiąt dziewięć złotych (00/100 groszy)</v>
+      <c r="D17" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F17" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1105,16 +1199,16 @@
       <c r="C18" s="4">
         <v>100</v>
       </c>
-      <c r="D18" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Sto złotych (00/100 groszy)</v>
+      <c r="D18" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F18" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1127,16 +1221,16 @@
       <c r="C19" s="10">
         <v>200</v>
       </c>
-      <c r="D19" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwieście złotych (00/100 groszy)</v>
+      <c r="D19" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F19" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1149,16 +1243,16 @@
       <c r="C20" s="4">
         <v>213</v>
       </c>
-      <c r="D20" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwieście trzynaście złotych (00/100 groszy)</v>
+      <c r="D20" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F20" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F20" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1171,16 +1265,16 @@
       <c r="C21" s="10">
         <v>999</v>
       </c>
-      <c r="D21" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziewięćset dziewięćdziesiąt dziewięć złotych (00/100 groszy)</v>
+      <c r="D21" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F21" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1193,16 +1287,16 @@
       <c r="C22" s="4">
         <v>1000</v>
       </c>
-      <c r="D22" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Tysiąc złotych (00/100 groszy)</v>
+      <c r="D22" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F22" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F22" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1215,16 +1309,16 @@
       <c r="C23" s="10">
         <v>2000</v>
       </c>
-      <c r="D23" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwa tysiące złotych (00/100 groszy)</v>
+      <c r="D23" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F23" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1237,16 +1331,16 @@
       <c r="C24" s="4">
         <v>5000</v>
       </c>
-      <c r="D24" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Pięć tysięcy złotych (00/100 groszy)</v>
+      <c r="D24" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F24" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1259,16 +1353,16 @@
       <c r="C25" s="10">
         <v>11000</v>
       </c>
-      <c r="D25" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Jedenaście tysięcy złotych (00/100 groszy)</v>
+      <c r="D25" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F25" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1281,16 +1375,16 @@
       <c r="C26" s="4">
         <v>12000</v>
       </c>
-      <c r="D26" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwanaście tysięcy złotych (00/100 groszy)</v>
+      <c r="D26" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F26" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1303,16 +1397,16 @@
       <c r="C27" s="10">
         <v>21000</v>
       </c>
-      <c r="D27" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwadzieścia jeden tysięcy złotych (00/100 groszy)</v>
+      <c r="D27" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F27" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F27" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1325,16 +1419,16 @@
       <c r="C28" s="4">
         <v>22000</v>
       </c>
-      <c r="D28" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwadzieścia dwa tysiące złotych (00/100 groszy)</v>
+      <c r="D28" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F28" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F28" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1347,16 +1441,16 @@
       <c r="C29" s="10">
         <v>1234</v>
       </c>
-      <c r="D29" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Tysiąc dwieście trzydzieści cztery złote (00/100 groszy)</v>
+      <c r="D29" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F29" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F29" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1369,16 +1463,16 @@
       <c r="C30" s="4">
         <v>1000000</v>
       </c>
-      <c r="D30" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Jeden milion złotych (00/100 groszy)</v>
+      <c r="D30" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F30" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F30" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1391,16 +1485,16 @@
       <c r="C31" s="10">
         <v>2000000</v>
       </c>
-      <c r="D31" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwa miliony złotych (00/100 groszy)</v>
+      <c r="D31" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F31" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F31" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1413,16 +1507,16 @@
       <c r="C32" s="4">
         <v>5000000</v>
       </c>
-      <c r="D32" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Pięć milionów złotych (00/100 groszy)</v>
+      <c r="D32" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F32" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F32" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1435,16 +1529,16 @@
       <c r="C33" s="10">
         <v>11000000</v>
       </c>
-      <c r="D33" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Jedenaście milionów złotych (00/100 groszy)</v>
+      <c r="D33" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F33" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F33" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1457,16 +1551,16 @@
       <c r="C34" s="4">
         <v>0.01</v>
       </c>
-      <c r="D34" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Zero złotych (01/100 groszy)</v>
+      <c r="D34" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F34" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F34" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1479,16 +1573,16 @@
       <c r="C35" s="10">
         <v>0.99</v>
       </c>
-      <c r="D35" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Zero złotych (99/100 groszy)</v>
+      <c r="D35" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F35" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F35" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1501,16 +1595,16 @@
       <c r="C36" s="4">
         <v>1.01</v>
       </c>
-      <c r="D36" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Jeden złoty (01/100 groszy)</v>
+      <c r="D36" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F36" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F36" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1523,16 +1617,16 @@
       <c r="C37" s="10">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D37" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Jeden złoty (10/100 groszy)</v>
+      <c r="D37" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F37" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F37" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1545,16 +1639,16 @@
       <c r="C38" s="4">
         <v>1234.67</v>
       </c>
-      <c r="D38" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Tysiąc dwieście trzydzieści cztery złote (67/100 groszy)</v>
+      <c r="D38" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F38" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F38" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1567,16 +1661,16 @@
       <c r="C39" s="10">
         <v>1.9990000000000001</v>
       </c>
-      <c r="D39" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Dwa złote (00/100 groszy)</v>
+      <c r="D39" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F39" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1587,18 +1681,18 @@
         <v>51</v>
       </c>
       <c r="C40" s="4">
-        <v>0.01</v>
-      </c>
-      <c r="D40" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Zero złotych (01/100 groszy)</v>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D40" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F40" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F40" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1611,16 +1705,16 @@
       <c r="C41" s="10">
         <v>999999999.99000001</v>
       </c>
-      <c r="D41" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Dziewięćset dziewięćdziesiąt dziewięć milionów dziewięćset dziewięćdziesiąt dziewięć tysięcy dziewięćset dziewięćdziesiąt dziewięć złotych (99/100 groszy)</v>
+      <c r="D41" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F41" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F41" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1633,16 +1727,16 @@
       <c r="C42" s="4">
         <v>-1</v>
       </c>
-      <c r="D42" s="23" t="str">
-        <f t="shared" si="0"/>
-        <v>Blad: ujemna liczba</v>
+      <c r="D42" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F42" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F42" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1655,41 +1749,1076 @@
       <c r="C43" s="10">
         <v>1000000000</v>
       </c>
-      <c r="D43" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Blad: liczba zbyt duza (max 999 999 999,99)</v>
+      <c r="D43" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F43" s="11" t="str">
-        <f t="shared" si="1"/>
-        <v>✅ OK</v>
+      <c r="F43" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="18" t="s">
+      <c r="A44" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="12">
-        <f>COUNTIF(F4:F43,"✅ OK")</f>
-        <v>40</v>
-      </c>
-      <c r="E44" s="13" t="s">
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="13">
+        <f ca="1">COUNTIF(F4:F43,"✅ OK")</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F44" s="14">
-        <f>COUNTIF(F4:F43,"❌ SPRAWDŹ")</f>
+      <c r="F44" s="15">
+        <f ca="1">COUNTIF(F4:F43,"❌ SPRAWDŹ")</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Arkusz2"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+    </row>
+    <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="e">
+        <f t="shared" ref="D4:D15" ca="1" si="0">PL_TEKST(C4,"EUR")</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="7" t="e">
+        <f t="shared" ref="F4:F15" ca="1" si="1">IF(D4=E4,"✅ OK","❌ SPRAWDŹ")</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="10">
+        <v>2</v>
+      </c>
+      <c r="D5" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10">
+        <v>11</v>
+      </c>
+      <c r="D7" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="10">
+        <v>21</v>
+      </c>
+      <c r="D9" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="4">
+        <v>100</v>
+      </c>
+      <c r="D10" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D11" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2000</v>
+      </c>
+      <c r="D12" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="10">
+        <v>1234.67</v>
+      </c>
+      <c r="D13" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="D14" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="10">
+        <v>0</v>
+      </c>
+      <c r="D15" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="13">
+        <f ca="1">COUNTIF(F4:F15,"✅ OK")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="15">
+        <f ca="1">COUNTIF(F4:F15,"❌ SPRAWDŹ")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Arkusz3"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+    </row>
+    <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="e">
+        <f t="shared" ref="D4:D15" ca="1" si="0">PL_TEKST(C4,"USD")</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="7" t="e">
+        <f t="shared" ref="F4:F15" ca="1" si="1">IF(D4=E4,"✅ OK","❌ SPRAWDŹ")</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="10">
+        <v>2</v>
+      </c>
+      <c r="D5" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10">
+        <v>11</v>
+      </c>
+      <c r="D7" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="10">
+        <v>21</v>
+      </c>
+      <c r="D9" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="4">
+        <v>100</v>
+      </c>
+      <c r="D10" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D11" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2000</v>
+      </c>
+      <c r="D12" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="10">
+        <v>1234.67</v>
+      </c>
+      <c r="D13" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="D14" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="10">
+        <v>0</v>
+      </c>
+      <c r="D15" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="13">
+        <f ca="1">COUNTIF(F4:F15,"✅ OK")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="15">
+        <f ca="1">COUNTIF(F4:F15,"❌ SPRAWDŹ")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Arkusz4"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+    </row>
+    <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="e">
+        <f t="shared" ref="D4:D15" ca="1" si="0">PL_TEKST(C4,"GBP")</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="7" t="e">
+        <f t="shared" ref="F4:F15" ca="1" si="1">IF(D4=E4,"✅ OK","❌ SPRAWDŹ")</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="10">
+        <v>2</v>
+      </c>
+      <c r="D5" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10">
+        <v>11</v>
+      </c>
+      <c r="D7" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="4">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="10">
+        <v>21</v>
+      </c>
+      <c r="D9" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F9" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="4">
+        <v>100</v>
+      </c>
+      <c r="D10" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F10" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D11" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F11" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2000</v>
+      </c>
+      <c r="D12" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="10">
+        <v>1234.67</v>
+      </c>
+      <c r="D13" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="D14" s="5" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="7" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="10">
+        <v>0</v>
+      </c>
+      <c r="D15" s="11" t="e">
+        <f t="shared" ca="1" si="0"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="12" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="13">
+        <f ca="1">COUNTIF(F4:F15,"✅ OK")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="15">
+        <f ca="1">COUNTIF(F4:F15,"❌ SPRAWDŹ")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>